<commit_message>
feat: new preprocess dataset and analysis code
</commit_message>
<xml_diff>
--- a/data/Labeled Questions and Answers.xlsx
+++ b/data/Labeled Questions and Answers.xlsx
@@ -449,7 +449,7 @@
         <v>none</v>
       </c>
       <c r="F2" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G2" t="str">
         <v>None</v>
@@ -1434,7 +1434,7 @@
         <v>none</v>
       </c>
       <c r="F22" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G22" t="str">
         <v>None found.</v>
@@ -1537,7 +1537,7 @@
         <v>no</v>
       </c>
       <c r="F24" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G24" t="str" xml:space="preserve">
         <v xml:space="preserve">None. Large deposits are sourced as account transfers:
@@ -1581,7 +1581,7 @@
         <v>none</v>
       </c>
       <c r="F25" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G25" t="str">
         <v>None noted.</v>
@@ -2248,7 +2248,7 @@
         <v>none</v>
       </c>
       <c r="F42" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G42" t="str">
         <v>None noted.</v>
@@ -2312,7 +2312,7 @@
         <v>none</v>
       </c>
       <c r="F44" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G44" t="str">
         <v>None noted.</v>
@@ -2348,7 +2348,7 @@
         <v>none</v>
       </c>
       <c r="F45" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G45" t="str">
         <v>None noted.</v>
@@ -2414,7 +2414,7 @@
         <v>none</v>
       </c>
       <c r="F47" t="str">
-        <v>none</v>
+        <v>id_list</v>
       </c>
       <c r="G47" t="str">
         <v>[SOLO transaction parsing is wrong here, treated a supplementary bank statement as a new one]</v>

</xml_diff>